<commit_message>
Add article subtitles and feedback to featured articles
Import each article's intro lead as a subtitle section (single title)
flush under the hero, styled like the source with Zilla Slab Light.
Content List teasers read the subtitle from that section and look up
referenced pages in the right place for author, preview and publish.
Featured articles also get the Feedback block, as on the source.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-hero.report.xlsx
+++ b/tools/importer/reports/import-article-hero.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="79">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,7 +19,7 @@
     <t>blocks</t>
   </si>
   <si>
-    <t>contentListMore</t>
+    <t>damImages</t>
   </si>
   <si>
     <t>heroImages</t>
@@ -31,6 +31,9 @@
     <t>status</t>
   </si>
   <si>
+    <t>subtitle</t>
+  </si>
+  <si>
     <t>template</t>
   </si>
   <si>
@@ -49,10 +52,10 @@
     <t>["hero","cards","columns","feedback"]</t>
   </si>
   <si>
-    <t>Featured: https://www.doc.govt.nz/footer-links/new-on-the-site/; Media releases: https://www.doc.govt.nz/news/media-releases/2026-media-releases/</t>
-  </si>
-  <si>
-    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/9b48a55da5974906b6d65a89fb9d5d06/kura-tawhiti-hero.jpg -&gt; /content/dam/nzdoc/heros/kura-tawhiti-hero.jpg</t>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/9b48a55da5974906b6d65a89fb9d5d06/kura-tawhiti-hero.jpg -&gt; /content/dam/nzdoc/heros/kura-tawhiti-hero.jpg; https://www.doc.govt.nz/thumbs/gallery/contentassets/a8cf8502518043808b916575ca1bb512/denniston-hero.jpg -&gt; /content/dam/nzdoc/heros/denniston-hero.jpg; https://i0.wp.com/blog.doc.govt.nz/wp-content/uploads/2026/09/black-robin-invertebrate-leon-everett-1-e1788825954346.jpg?w=200 -&gt; /content/dam/nzdoc/blogs/2026/black-robin-invertebrate-leon-everett-1-e1788825954346.jpg</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>index</t>
@@ -64,7 +67,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-28T02:52:36.786Z</t>
+    <t>2026-09-28T03:31:15.762Z</t>
   </si>
   <si>
     <t>EMA: Department of Conservation</t>
@@ -76,76 +79,88 @@
     <t>news/issues/bird-flu-updates.report.json</t>
   </si>
   <si>
+    <t>["breadcrumb","hero","feedback"]</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/globalassets/images/nature/native-animals/birds/brown-skua/brown-skua-1920.jpg -&gt; /content/dam/nzdoc/heros/brown-skua-1920.jpg</t>
+  </si>
+  <si>
+    <t>news/issues/bird-flu-updates</t>
+  </si>
+  <si>
+    <t>H5 bird flu (H5N1 avian influenza) has been detected in New Zealand.</t>
+  </si>
+  <si>
+    <t>article-hero</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:53:56.352Z</t>
+  </si>
+  <si>
+    <t>EMA: Bird flu updates: Issues</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/news/issues/bird-flu-updates/</t>
+  </si>
+  <si>
+    <t>about-us/our-role/managing-conservation/conservation-amendment-bill.report.json</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/59e382809add463ea8fa893707db334d/whakatane-hero.jpg -&gt; /content/dam/nzdoc/heros/whakatane-hero.jpg</t>
+  </si>
+  <si>
+    <t>about-us/our-role/managing-conservation/conservation-amendment-bill</t>
+  </si>
+  <si>
+    <t>The Conservation Amendment Bill aims to modernise the way conservation land is managed, support economic growth, and deliver stronger conservation outcomes.</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:54:09.373Z</t>
+  </si>
+  <si>
+    <t>EMA: Conservation Amendment Bill: Managing conservation</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/about-us/our-role/managing-conservation/conservation-amendment-bill/</t>
+  </si>
+  <si>
+    <t>news/events/national-events/national-wild-goat-hunting-competition.report.json</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/f7be0a20cbaa45f1b78b2d52b6d366b2/national-wild-goat-competition-2026-1920.jpg -&gt; /content/dam/nzdoc/heros/national-wild-goat-competition-2026-1920.jpg</t>
+  </si>
+  <si>
+    <t>news/events/national-events/national-wild-goat-hunting-competition</t>
+  </si>
+  <si>
+    <t>Turn your wild goat hunt – whether it's your first or your fourth, solo or with mates – into meaningful action. Help reduce pressure on New Zealand's landscapes and go in the draw to win.</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:54:14.897Z</t>
+  </si>
+  <si>
+    <t>EMA: National Wild Goat Hunting Competition 2026</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/news/events/national-events/national-wild-goat-hunting-competition/</t>
+  </si>
+  <si>
+    <t>news/media-releases/2026-media-releases/4wd-group-plants-native-trees-to-fix-damage.report.json</t>
+  </si>
+  <si>
     <t>["breadcrumb","hero"]</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>https://www.doc.govt.nz/thumbs/hero/globalassets/images/nature/native-animals/birds/brown-skua/brown-skua-1920.jpg -&gt; /content/dam/nzdoc/heros/brown-skua-1920.jpg</t>
-  </si>
-  <si>
-    <t>news/issues/bird-flu-updates</t>
-  </si>
-  <si>
-    <t>article-hero</t>
-  </si>
-  <si>
-    <t>2026-09-28T03:05:43.233Z</t>
-  </si>
-  <si>
-    <t>EMA: Bird flu updates: Issues</t>
-  </si>
-  <si>
-    <t>https://www.doc.govt.nz/news/issues/bird-flu-updates/</t>
-  </si>
-  <si>
-    <t>about-us/our-role/managing-conservation/conservation-amendment-bill.report.json</t>
-  </si>
-  <si>
-    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/59e382809add463ea8fa893707db334d/whakatane-hero.jpg -&gt; /content/dam/nzdoc/heros/whakatane-hero.jpg</t>
-  </si>
-  <si>
-    <t>about-us/our-role/managing-conservation/conservation-amendment-bill</t>
-  </si>
-  <si>
-    <t>2026-09-28T03:05:57.831Z</t>
-  </si>
-  <si>
-    <t>EMA: Conservation Amendment Bill: Managing conservation</t>
-  </si>
-  <si>
-    <t>https://www.doc.govt.nz/about-us/our-role/managing-conservation/conservation-amendment-bill/</t>
-  </si>
-  <si>
-    <t>news/events/national-events/national-wild-goat-hunting-competition.report.json</t>
-  </si>
-  <si>
-    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/f7be0a20cbaa45f1b78b2d52b6d366b2/national-wild-goat-competition-2026-1920.jpg -&gt; /content/dam/nzdoc/heros/national-wild-goat-competition-2026-1920.jpg</t>
-  </si>
-  <si>
-    <t>news/events/national-events/national-wild-goat-hunting-competition</t>
-  </si>
-  <si>
-    <t>2026-09-28T03:14:05.267Z</t>
-  </si>
-  <si>
-    <t>EMA: National Wild Goat Hunting Competition 2026</t>
-  </si>
-  <si>
-    <t>https://www.doc.govt.nz/news/events/national-events/national-wild-goat-hunting-competition/</t>
-  </si>
-  <si>
-    <t>news/media-releases/2026-media-releases/4wd-group-plants-native-trees-to-fix-damage.report.json</t>
-  </si>
-  <si>
     <t>https://www.doc.govt.nz/thumbs/hero/contentassets/6bd3432a1fe849b3848184b73ccc07b6/planting-with-damage-in-background1920.jpg -&gt; /content/dam/nzdoc/heros/planting-with-damage-in-background1920.jpg</t>
   </si>
   <si>
     <t>news/media-releases/2026-media-releases/4wd-group-plants-native-trees-to-fix-damage</t>
   </si>
   <si>
-    <t>2026-09-28T03:06:25.267Z</t>
+    <t>A four-wheel drive (4WD) club has joined forces with the Department of Conservation to fund and plant native shrubs and trees to help cover damage done by vehicles.</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:54:33.072Z</t>
   </si>
   <si>
     <t>EMA: 4WD group plants native trees to fix damage</t>
@@ -160,7 +175,10 @@
     <t>news/media-releases/2026-media-releases/funding-boost-for-bird-flu-surveillance</t>
   </si>
   <si>
-    <t>2026-09-28T03:06:12.822Z</t>
+    <t>The government is boosting support for wildlife care facilities because of their key role in New Zealand’s bird flu surveillance and response, Conservation Minister Tama Potaka and Biosecurity Minister Andrew Hoggard say.</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:54:21.591Z</t>
   </si>
   <si>
     <t>EMA: Funding boost for bird flu surveillance: Media release 24 September 2026</t>
@@ -178,7 +196,10 @@
     <t>news/media-releases/2026-media-releases/government-invests-in-cleaning-up-contaminated-crown-land</t>
   </si>
   <si>
-    <t>2026-09-28T03:06:18.888Z</t>
+    <t>The Government is taking a practical step to address contaminated sites on Crown-owned land.</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:54:27.239Z</t>
   </si>
   <si>
     <t>EMA: Government invests in cleaning up contaminated Crown land: Media release 23 September 2026</t>
@@ -196,7 +217,10 @@
     <t>news/media-releases/2026-media-releases/toxoplasmosis-confirmed-as-cause-of-death-of-pregnant-hectors-dolphin</t>
   </si>
   <si>
-    <t>2026-09-28T03:06:32.869Z</t>
+    <t>DOC has confirmed toxoplasmosis was the cause of death of a pregnant Hector’s dolphin found at Invercargill’s Oreti Beach last month.</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:54:38.824Z</t>
   </si>
   <si>
     <t>EMA: Toxoplasmosis confirmed as cause of death of pregnant Hector’s dolphin: Media release 22 September 2026</t>
@@ -214,7 +238,10 @@
     <t>parks-and-recreation/things-to-do/fishing/whitebaiting</t>
   </si>
   <si>
-    <t>2026-09-28T03:05:51.019Z</t>
+    <t>The whitebait fishing season is open. Find out when, where and how to fish for whitebait in New Zealand and the Chatham Islands.</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:54:02.394Z</t>
   </si>
   <si>
     <t>EMA: Whitebaiting: Things to do</t>
@@ -609,18 +636,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="39" customWidth="1"/>
     <col min="3" max="5" width="50" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="26" customWidth="1"/>
-    <col min="9" max="10" width="50" customWidth="1"/>
+    <col min="7" max="7" width="50" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="11" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -651,28 +679,31 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" t="s">
         <v>14</v>
-      </c>
-      <c r="F2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" t="s">
-        <v>16</v>
       </c>
       <c r="H2" t="s">
         <v>17</v>
@@ -683,16 +714,19 @@
       <c r="J2" t="s">
         <v>19</v>
       </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
         <v>23</v>
@@ -701,7 +735,7 @@
         <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G3" t="s">
         <v>25</v>
@@ -715,233 +749,257 @@
       <c r="J3" t="s">
         <v>28</v>
       </c>
+      <c r="K3" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
         <v>22</v>
       </c>
-      <c r="D4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4" t="s">
-        <v>32</v>
-      </c>
-      <c r="I4" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" t="s">
-        <v>34</v>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" t="s">
+        <v>41</v>
+      </c>
+      <c r="J5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K5" t="s">
+        <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" t="s">
-        <v>38</v>
-      </c>
-      <c r="I5" t="s">
-        <v>39</v>
-      </c>
-      <c r="J5" t="s">
-        <v>40</v>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K6" t="s">
+        <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E6" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I6" t="s">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" t="s">
         <v>45</v>
       </c>
-      <c r="J6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" t="s">
-        <v>21</v>
-      </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
       </c>
       <c r="E7" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G7" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="H7" t="s">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="I7" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="J7" t="s">
-        <v>51</v>
+        <v>56</v>
+      </c>
+      <c r="K7" t="s">
+        <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
+        <v>61</v>
+      </c>
+      <c r="H8" t="s">
+        <v>26</v>
+      </c>
+      <c r="I8" t="s">
+        <v>62</v>
+      </c>
+      <c r="J8" t="s">
+        <v>63</v>
+      </c>
+      <c r="K8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" t="s">
+        <v>68</v>
+      </c>
+      <c r="H9" t="s">
+        <v>26</v>
+      </c>
+      <c r="I9" t="s">
+        <v>69</v>
+      </c>
+      <c r="J9" t="s">
+        <v>70</v>
+      </c>
+      <c r="K9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" t="s">
         <v>22</v>
       </c>
-      <c r="D8" t="s">
-        <v>53</v>
-      </c>
-      <c r="E8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8" t="s">
-        <v>55</v>
-      </c>
-      <c r="I8" t="s">
-        <v>56</v>
-      </c>
-      <c r="J8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" t="s">
-        <v>59</v>
-      </c>
-      <c r="E9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" t="s">
-        <v>25</v>
-      </c>
-      <c r="H9" t="s">
-        <v>61</v>
-      </c>
-      <c r="I9" t="s">
-        <v>62</v>
-      </c>
-      <c r="J9" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>64</v>
-      </c>
-      <c r="B10" t="s">
-        <v>21</v>
-      </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="F10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G10" t="s">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="I10" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="J10" t="s">
-        <v>69</v>
+        <v>77</v>
+      </c>
+      <c r="K10" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Migrate Short Walks overview: text and video columns
Import the Short Walks landing page (breadcrumb, hero, subtitle,
overview columns, feedback). The overview text goes in the first
column and the YouTube video in an Embed placed into the second
column when rendering; Embed is allowed in columns in the editor.
The hero import skips overlaid programme logos. Panel body copy
uses the source styles, plain buttons in content read as links, and
the subtitle is the title that opens the section under the hero.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-hero.report.xlsx
+++ b/tools/importer/reports/import-article-hero.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="87">
   <si>
     <t>_reportFile</t>
   </si>
@@ -248,6 +248,30 @@
   </si>
   <si>
     <t>https://www.doc.govt.nz/parks-and-recreation/things-to-do/fishing/whitebaiting/</t>
+  </si>
+  <si>
+    <t>parks-and-recreation/things-to-do/walking-and-tramping/short-walks.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb","hero","columns","feedback"]</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/a8cf8502518043808b916575ca1bb512/denniston-hero.jpg -&gt; /content/dam/nzdoc/heros/denniston-hero.jpg</t>
+  </si>
+  <si>
+    <t>parks-and-recreation/things-to-do/walking-and-tramping/short-walks</t>
+  </si>
+  <si>
+    <t>Discover some of our best short walks. They’re easy to get to and great for families – there’s something for everyone.</t>
+  </si>
+  <si>
+    <t>2026-09-29T03:02:53.982Z</t>
+  </si>
+  <si>
+    <t>EMA: Short Walks: Walking and tramping</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/parks-and-recreation/things-to-do/walking-and-tramping/short-walks/</t>
   </si>
 </sst>
 </file>
@@ -636,11 +660,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
-    <col min="2" max="2" width="39" customWidth="1"/>
+    <col min="2" max="2" width="44" customWidth="1"/>
     <col min="3" max="5" width="50" customWidth="1"/>
     <col min="7" max="7" width="50" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
@@ -998,6 +1022,41 @@
         <v>78</v>
       </c>
     </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" t="s">
+        <v>81</v>
+      </c>
+      <c r="E11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" t="s">
+        <v>83</v>
+      </c>
+      <c r="H11" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" t="s">
+        <v>84</v>
+      </c>
+      <c r="J11" t="s">
+        <v>85</v>
+      </c>
+      <c r="K11" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Point links to migrated pages at the migrated copy
A new import transformer rewrites links to source pages that are
already migrated (every URL in page-templates.json) to their AEM page
path, like the content references; other links keep pointing at the
source site. The homepage Short Walks card now links to the migrated
Short Walks page.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-hero.report.xlsx
+++ b/tools/importer/reports/import-article-hero.report.xlsx
@@ -67,7 +67,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-28T03:31:15.762Z</t>
+    <t>2026-09-29T03:18:55.011Z</t>
   </si>
   <si>
     <t>EMA: Department of Conservation</t>
@@ -94,7 +94,7 @@
     <t>article-hero</t>
   </si>
   <si>
-    <t>2026-09-28T03:53:56.352Z</t>
+    <t>2026-09-29T03:19:03.033Z</t>
   </si>
   <si>
     <t>EMA: Bird flu updates: Issues</t>
@@ -115,7 +115,7 @@
     <t>The Conservation Amendment Bill aims to modernise the way conservation land is managed, support economic growth, and deliver stronger conservation outcomes.</t>
   </si>
   <si>
-    <t>2026-09-28T03:54:09.373Z</t>
+    <t>2026-09-29T03:19:16.392Z</t>
   </si>
   <si>
     <t>EMA: Conservation Amendment Bill: Managing conservation</t>
@@ -136,7 +136,7 @@
     <t>Turn your wild goat hunt – whether it's your first or your fourth, solo or with mates – into meaningful action. Help reduce pressure on New Zealand's landscapes and go in the draw to win.</t>
   </si>
   <si>
-    <t>2026-09-28T03:54:14.897Z</t>
+    <t>2026-09-29T03:19:24.194Z</t>
   </si>
   <si>
     <t>EMA: National Wild Goat Hunting Competition 2026</t>
@@ -160,7 +160,7 @@
     <t>A four-wheel drive (4WD) club has joined forces with the Department of Conservation to fund and plant native shrubs and trees to help cover damage done by vehicles.</t>
   </si>
   <si>
-    <t>2026-09-28T03:54:33.072Z</t>
+    <t>2026-09-29T03:19:42.140Z</t>
   </si>
   <si>
     <t>EMA: 4WD group plants native trees to fix damage</t>
@@ -178,7 +178,7 @@
     <t>The government is boosting support for wildlife care facilities because of their key role in New Zealand’s bird flu surveillance and response, Conservation Minister Tama Potaka and Biosecurity Minister Andrew Hoggard say.</t>
   </si>
   <si>
-    <t>2026-09-28T03:54:21.591Z</t>
+    <t>2026-09-29T03:19:30.980Z</t>
   </si>
   <si>
     <t>EMA: Funding boost for bird flu surveillance: Media release 24 September 2026</t>
@@ -199,7 +199,7 @@
     <t>The Government is taking a practical step to address contaminated sites on Crown-owned land.</t>
   </si>
   <si>
-    <t>2026-09-28T03:54:27.239Z</t>
+    <t>2026-09-29T03:19:36.448Z</t>
   </si>
   <si>
     <t>EMA: Government invests in cleaning up contaminated Crown land: Media release 23 September 2026</t>
@@ -220,7 +220,7 @@
     <t>DOC has confirmed toxoplasmosis was the cause of death of a pregnant Hector’s dolphin found at Invercargill’s Oreti Beach last month.</t>
   </si>
   <si>
-    <t>2026-09-28T03:54:38.824Z</t>
+    <t>2026-09-29T03:19:49.230Z</t>
   </si>
   <si>
     <t>EMA: Toxoplasmosis confirmed as cause of death of pregnant Hector’s dolphin: Media release 22 September 2026</t>
@@ -241,7 +241,7 @@
     <t>The whitebait fishing season is open. Find out when, where and how to fish for whitebait in New Zealand and the Chatham Islands.</t>
   </si>
   <si>
-    <t>2026-09-28T03:54:02.394Z</t>
+    <t>2026-09-29T03:19:09.164Z</t>
   </si>
   <si>
     <t>EMA: Whitebaiting: Things to do</t>
@@ -265,7 +265,7 @@
     <t>Discover some of our best short walks. They’re easy to get to and great for families – there’s something for everyone.</t>
   </si>
   <si>
-    <t>2026-09-29T03:02:53.982Z</t>
+    <t>2026-09-29T03:20:14.137Z</t>
   </si>
   <si>
     <t>EMA: Short Walks: Walking and tramping</t>

</xml_diff>